<commit_message>
model 2020 adjustments and python files
</commit_message>
<xml_diff>
--- a/model_fitting/2020/patches 2020/results_chisquare.xlsx
+++ b/model_fitting/2020/patches 2020/results_chisquare.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -551,19 +551,40 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>multiple_birth</t>
+          <t>multiple_birth_binary</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>402.85</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>province_mother</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1539.88</v>
+      </c>
+      <c r="C8" t="n">
+        <v>64</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>Yes ***</t>
         </is>

</xml_diff>